<commit_message>
Update grid data and add rendered images
Latest property grid with 17 properties x 10 protocols.
Add high-res PNG renders of both grids.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/privacy_feature_grid.xlsx
+++ b/privacy_feature_grid.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="007A7490"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="000C0A18"/>
       <sz val="10"/>
@@ -75,6 +81,12 @@
       <name val="Arial"/>
       <color rgb="008B5E3C"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B4420"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -156,12 +168,6 @@
       <color rgb="007A7490"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="006B4420"/>
-      <sz val="11"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -236,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -245,7 +251,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -254,11 +260,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -266,14 +272,14 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -281,33 +287,39 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -317,59 +329,59 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -738,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -866,8 +878,8 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Compliance
-(viewing keys)</t>
+          <t>Selective
+disclosure</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -896,8 +908,8 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Fast proof
-generation</t>
+          <t>End-to-end
+transaction time</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -908,8 +920,8 @@
       </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
-          <t>Rich client-side
-proving</t>
+          <t>Programmable
+privacy</t>
         </is>
       </c>
       <c r="N5" s="8" t="inlineStr">
@@ -948,1038 +960,1119 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>one pool hides
+all token types</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>ZK property
+formally proven</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>one key, no
+secrets to lose</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>find your
+funds fast</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>reveal only
+what you choose</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>no ceremony,
+no trust needed</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>safe from
+quantum computers</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>anyone can
+verify the chain</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>go private or
+public in seconds</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>proof +
+confirmation speed</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>high throughput,
+low cost</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>complex DeFi ops,
+fully private</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>works with
+existing protocols</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>real users,
+real liquidity</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>runs on
+EVM chains</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>multisig, recovery,
+session keys</t>
+        </is>
+      </c>
+      <c r="R6" s="9" t="inlineStr">
+        <is>
+          <t>sign with
+Ledger/Trezor</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>STRK20s (Starknet)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P6" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q6" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R6" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S6" s="12" t="inlineStr">
-        <is>
-          <t>14/17</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>(✓)²⁴</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q7" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S7" s="14" t="inlineStr">
+        <is>
+          <t>13.5/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Zcash</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>(✓)²</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K7" s="16" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>(✓)¹⁸</t>
         </is>
       </c>
-      <c r="L7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O7" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R7" s="16" t="inlineStr">
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R8" s="18" t="inlineStr">
         <is>
           <t>(✓)¹⁴</t>
         </is>
       </c>
-      <c r="S7" s="17" t="inlineStr">
+      <c r="S8" s="19" t="inlineStr">
         <is>
           <t>4.5/17</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Monero</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>(✓)¹</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>(✓)²¹</t>
         </is>
       </c>
-      <c r="K8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O8" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q8" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R8" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="S8" s="22" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O9" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q9" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R9" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="S9" s="24" t="inlineStr">
         <is>
           <t>4/17</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Aztec</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>(✓)⁴</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J9" s="16" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
         <is>
           <t>(✓)²³</t>
         </is>
       </c>
-      <c r="K9" s="16" t="inlineStr">
+      <c r="K10" s="18" t="inlineStr">
         <is>
           <t>(✓)¹⁵</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
+      <c r="L10" s="18" t="inlineStr">
         <is>
           <t>(✓)⁸</t>
         </is>
       </c>
-      <c r="M9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N9" s="16" t="inlineStr">
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>(✓)³</t>
         </is>
       </c>
-      <c r="O9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="P9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q9" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="R9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S9" s="17" t="inlineStr">
+      <c r="O10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="P10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S10" s="19" t="inlineStr">
         <is>
           <t>8.5/17</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Aleo</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F10" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="inlineStr">
         <is>
           <t>(✓)¹⁶</t>
         </is>
       </c>
-      <c r="L10" s="20" t="inlineStr">
+      <c r="L11" s="22" t="inlineStr">
         <is>
           <t>(✓)¹³</t>
         </is>
       </c>
-      <c r="M10" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O10" s="20" t="inlineStr">
+      <c r="M11" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O11" s="22" t="inlineStr">
         <is>
           <t>(✓)¹²</t>
         </is>
       </c>
-      <c r="P10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R10" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S10" s="22" t="inlineStr">
+      <c r="P11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R11" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S11" s="24" t="inlineStr">
         <is>
           <t>4.5/17</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Railgun</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P11" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Q11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S11" s="17" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S12" s="19" t="inlineStr">
         <is>
           <t>6/17</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Solana confidential</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>(✓)⁵</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O12" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q12" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R12" s="20" t="inlineStr">
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O13" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q13" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R13" s="22" t="inlineStr">
         <is>
           <t>(✓)¹⁷</t>
         </is>
       </c>
-      <c r="S12" s="22" t="inlineStr">
+      <c r="S13" s="24" t="inlineStr">
         <is>
           <t>3/17</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Canton</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L13" s="16" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
         <is>
           <t>(✓)¹¹</t>
         </is>
       </c>
-      <c r="M13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N13" s="16" t="inlineStr">
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
         <is>
           <t>(✓)¹⁰</t>
         </is>
       </c>
-      <c r="O13" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S13" s="17" t="inlineStr">
+      <c r="O14" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S14" s="19" t="inlineStr">
         <is>
           <t>4/17</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Tornado Cash</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="P14" s="21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Q14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R14" s="19" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S14" s="22" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="P15" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R15" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S15" s="24" t="inlineStr">
         <is>
           <t>2/17</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Zama (FHE)</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>(✓)⁷</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>(✓)⁶</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="O15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="P15" s="15" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Q15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="R15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="S15" s="17" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="P16" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="R16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S16" s="19" t="inlineStr">
         <is>
           <t>4/17</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>✓ = full capability</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>(✓) = capability with caveats (see footnotes)</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="25" t="inlineStr">
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="27" t="inlineStr">
         <is>
           <t>– = absent or not applicable</t>
         </is>
       </c>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
-      <c r="P17" s="3" t="n"/>
-      <c r="Q17" s="3" t="n"/>
-      <c r="R17" s="3" t="n"/>
-      <c r="S17" s="3" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="n"/>
+      <c r="P18" s="3" t="n"/>
+      <c r="Q18" s="3" t="n"/>
+      <c r="R18" s="3" t="n"/>
+      <c r="S18" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Footnotes</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
-      <c r="P19" s="3" t="n"/>
-      <c r="Q19" s="3" t="n"/>
-      <c r="R19" s="3" t="n"/>
-      <c r="S19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="27" t="inlineStr">
-        <is>
-          <t>¹  incoming transactions only. can’t reliably view outgoing or verify balance. all-or-nothing, no per-transaction selectivity</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
@@ -2002,9 +2095,9 @@
       <c r="S20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>²  Orchard pool only (since May 2022). Sapling pool still relies on a trusted setup ceremony</t>
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>¹  incoming transactions only. can’t reliably view outgoing or verify balance. all-or-nothing, no per-transaction selectivity</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
@@ -2027,9 +2120,9 @@
       <c r="S21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
-        <is>
-          <t>³  composable private/public functions exist, but within Aztec’s own nascent ecosystem. no existing DeFi protocols to compose with yet</t>
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>²  Orchard pool only (since May 2022). Sapling pool still relies on a trusted setup ceremony</t>
         </is>
       </c>
       <c r="B22" s="3" t="n"/>
@@ -2052,9 +2145,9 @@
       <c r="S22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
-        <is>
-          <t>⁴  tagging mechanism requires pre-registering senders. can’t discover notes from unknown senders</t>
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>³  composable private/public functions exist, but within Aztec’s own nascent ecosystem. no existing DeFi protocols to compose with yet</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
@@ -2077,9 +2170,9 @@
       <c r="S23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
-        <is>
-          <t>⁵  auditor_elgamal_pubkey exists in mint config, but the entire confidential transfer feature is currently disabled on mainnet pending security audit</t>
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>⁴  tagging mechanism requires pre-registering senders. can’t discover notes from unknown senders</t>
         </is>
       </c>
       <c r="B24" s="3" t="n"/>
@@ -2102,9 +2195,9 @@
       <c r="S24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
-        <is>
-          <t>⁶  TFHE is lattice-based (LWE hardness assumption), considered PQ-resistant but less battle-tested than hash-based approaches</t>
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>⁵  auditor_elgamal_pubkey exists in mint config, but the entire confidential transfer feature is currently disabled on mainnet pending security audit</t>
         </is>
       </c>
       <c r="B25" s="3" t="n"/>
@@ -2127,9 +2220,9 @@
       <c r="S25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
-        <is>
-          <t>⁷  confidential ERC-20s technically possible via fhEVM, but ecosystem is nascent with limited live deployments</t>
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>⁶  TFHE is lattice-based (LWE hardness assumption), considered PQ-resistant but less battle-tested than hash-based approaches</t>
         </is>
       </c>
       <c r="B26" s="3" t="n"/>
@@ -2152,9 +2245,9 @@
       <c r="S26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
-        <is>
-          <t>⁸  ZK rollup architecture is inherently scalable, but currently ~1 TPS in Alpha with 36–72s block times. targeting 3–4s by end of 2026</t>
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>⁷  confidential ERC-20s technically possible via fhEVM, but ecosystem is nascent with limited live deployments</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -2177,9 +2270,9 @@
       <c r="S27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="inlineStr">
-        <is>
-          <t>⁹  access-control privacy model (parties see only their part of a transaction). fundamentally different from ZK-based privacy: counterparties and validators see your data</t>
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>⁸  ZK rollup architecture is inherently scalable, but currently ~1 TPS in Alpha with 36–72s block times. targeting 3–4s by end of 2026</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -2202,9 +2295,9 @@
       <c r="S28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="inlineStr">
-        <is>
-          <t>¹⁰  DeFi exists within Canton’s own Daml ecosystem. requires Daml, a separate smart contract language. not composable with Ethereum/Starknet DeFi</t>
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>⁹  access-control privacy model (parties see only their part of a transaction). fundamentally different from ZK-based privacy: counterparties and validators see your data</t>
         </is>
       </c>
       <c r="B29" s="3" t="n"/>
@@ -2227,9 +2320,9 @@
       <c r="S29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="inlineStr">
-        <is>
-          <t>¹¹  horizontal scaling via network-of-networks. each node only processes its own transactions. claims no upper bound on TPS, but access-control privacy model</t>
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>¹⁰  DeFi exists within Canton’s own Daml ecosystem. requires Daml, a separate smart contract language. not composable with Ethereum/Starknet DeFi</t>
         </is>
       </c>
       <c r="B30" s="3" t="n"/>
@@ -2252,9 +2345,9 @@
       <c r="S30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr">
-        <is>
-          <t>¹²  mainnet since Sep 2024. USDCx with Circle launched Jan 2026. 350+ apps on testnet. but DeFi ecosystem still nascent</t>
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>¹¹  horizontal scaling via network-of-networks. each node only processes its own transactions. claims no upper bound on TPS, but access-control privacy model</t>
         </is>
       </c>
       <c r="B31" s="3" t="n"/>
@@ -2277,9 +2370,9 @@
       <c r="S31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="inlineStr">
-        <is>
-          <t>¹³  off-chain execution model enables scalable private computation, but no composability between private applications limits real-world DeFi throughput</t>
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>¹²  mainnet since Sep 2024. USDCx with Circle launched Jan 2026. 350+ apps on testnet. but DeFi ecosystem still nascent</t>
         </is>
       </c>
       <c r="B32" s="3" t="n"/>
@@ -2302,9 +2395,9 @@
       <c r="S32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="inlineStr">
-        <is>
-          <t>¹⁴  Trezor supports Orchard shielded transactions. Ledger supports transparent Zcash only</t>
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>¹³  off-chain execution model enables scalable private computation, but no composability between private applications limits real-world DeFi throughput</t>
         </is>
       </c>
       <c r="B33" s="3" t="n"/>
@@ -2327,9 +2420,9 @@
       <c r="S33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="inlineStr">
-        <is>
-          <t>¹⁵  PXE client-side proving works but proving times still being optimized. variable depending on circuit complexity</t>
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>¹⁴  Trezor supports Orchard shielded transactions. Ledger supports transparent Zcash only</t>
         </is>
       </c>
       <c r="B34" s="3" t="n"/>
@@ -2352,9 +2445,9 @@
       <c r="S34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="inlineStr">
-        <is>
-          <t>¹⁶  can outsource to Prover Market (Proof-as-a-Service). client-side proving possible but resource-intensive</t>
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>¹⁵  PXE client-side proving works but proving times still being optimized. variable depending on circuit complexity</t>
         </is>
       </c>
       <c r="B35" s="3" t="n"/>
@@ -2377,9 +2470,9 @@
       <c r="S35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="inlineStr">
-        <is>
-          <t>¹⁷  Ledger supports Solana but confidential transfer feature is currently disabled on mainnet</t>
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>¹⁶  can outsource to Prover Market (Proof-as-a-Service). client-side proving possible but resource-intensive</t>
         </is>
       </c>
       <c r="B36" s="3" t="n"/>
@@ -2402,9 +2495,9 @@
       <c r="S36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="inlineStr">
-        <is>
-          <t>¹⁸  Orchard proofs ~2–5s on modern hardware, but limited to simple shielded transfer logic</t>
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>¹⁷  Ledger supports Solana but confidential transfer feature is currently disabled on mainnet</t>
         </is>
       </c>
       <c r="B37" s="3" t="n"/>
@@ -2427,9 +2520,9 @@
       <c r="S37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="inlineStr">
-        <is>
-          <t>¹⁹  Bulletproofs+ for amount hiding are formally ZK, but core sender privacy relies on ring signatures which are a different cryptographic mechanism</t>
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>¹⁸  Orchard proofs ~2–5s on modern hardware, but limited to simple shielded transfer logic</t>
         </is>
       </c>
       <c r="B38" s="3" t="n"/>
@@ -2452,9 +2545,9 @@
       <c r="S38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="inlineStr">
-        <is>
-          <t>²⁰  Bulletproofs for range proofs are formally ZK, but scope is limited to amount hiding only</t>
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>¹⁹  Bulletproofs+ for amount hiding are formally ZK, but core sender privacy relies on ring signatures which are a different cryptographic mechanism</t>
         </is>
       </c>
       <c r="B39" s="3" t="n"/>
@@ -2477,9 +2570,9 @@
       <c r="S39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="inlineStr">
-        <is>
-          <t>²¹  always private by default. no shielding needed (instant opt-in), but no way to opt-out to a transparent state</t>
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>²⁰  Bulletproofs for range proofs are formally ZK, but scope is limited to amount hiding only</t>
         </is>
       </c>
       <c r="B40" s="3" t="n"/>
@@ -2502,9 +2595,9 @@
       <c r="S40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="inlineStr">
-        <is>
-          <t>²²  1-hour mandatory standby period after shielding before funds can be used privately (Private Proof of Innocence requirement)</t>
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>²¹  always private by default. no shielding needed (instant opt-in), but no way to opt-out to a transparent state</t>
         </is>
       </c>
       <c r="B41" s="3" t="n"/>
@@ -2527,9 +2620,9 @@
       <c r="S41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="inlineStr">
-        <is>
-          <t>²³  36–72s block times in Alpha. shielding speed will improve as block times target 3–4s by late 2026</t>
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>²²  1-hour mandatory standby period after shielding before funds can be used privately (Private Proof of Innocence requirement)</t>
         </is>
       </c>
       <c r="B42" s="3" t="n"/>
@@ -2551,8 +2644,58 @@
       <c r="R42" s="3" t="n"/>
       <c r="S42" s="3" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>²³  36–72s block times in Alpha. shielding speed will improve as block times target 3–4s by late 2026</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="3" t="n"/>
+      <c r="S43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>²⁴  ~5s end-to-end from user perspective, but proof runs on wallet operator backend (48-core machine). Zcash Zashi generates proofs directly on mobile in ~5s. for an apples-to-apples comparison, proof generation is not yet on consumer hardware. mobile proving on the roadmap</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="n"/>
+      <c r="N44" s="3" t="n"/>
+      <c r="O44" s="3" t="n"/>
+      <c r="P44" s="3" t="n"/>
+      <c r="Q44" s="3" t="n"/>
+      <c r="R44" s="3" t="n"/>
+      <c r="S44" s="3" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A42:S42"/>
     <mergeCell ref="N4:R4"/>
@@ -2561,10 +2704,11 @@
     <mergeCell ref="A32:S32"/>
     <mergeCell ref="A22:S22"/>
     <mergeCell ref="A35:S35"/>
-    <mergeCell ref="A20:S20"/>
     <mergeCell ref="A38:S38"/>
     <mergeCell ref="A29:S29"/>
+    <mergeCell ref="A43:S43"/>
     <mergeCell ref="A28:S28"/>
+    <mergeCell ref="A44:S44"/>
     <mergeCell ref="A40:S40"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="G4:I4"/>
@@ -2602,19 +2746,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>Definition &amp; Rationale</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>PRIVACY MODEL</t>
         </is>
@@ -2622,67 +2766,67 @@
       <c r="B2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="31" t="inlineStr">
         <is>
           <t>Multi-asset privacy pool</t>
         </is>
       </c>
-      <c r="B3" s="30" t="inlineStr">
+      <c r="B3" s="32" t="inlineStr">
         <is>
           <t>single pool supports multiple token types. observers can’t tell which token a note belongs to. STRK20s, Aztec, and Railgun have full multi-asset pools. Zama supports confidential ERC-20s via fhEVM but ecosystem is nascent. Aleo is asset-agnostic but each program has isolated state with no composability between private applications, so no unified pool. Zcash/Monero are single-asset. Tornado Cash had fragmented pools per token per amount. Canton uses access-control privacy, not a shielded pool model.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Formally ZK proofs</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="32" t="inlineStr">
         <is>
           <t>the proof system has the mathematical zero-knowledge property: the proof itself guarantees that no information about the secret data leaks to the verifier. This is distinct from privacy-as-UX. Many ZK rollups (including Starknet today) use validity proofs that prove correct execution but do not have the formal ZK property, meaning the proof could theoretically leak information about the underlying computation. Aztec’s CEO calls their architecture a ‘zk-zk rollup’: inner SNARKs (per-transaction) have the formal ZK property, outer SNARKs (rollup) also have it. Zcash (Groth16/Halo 2), Railgun (Groth16), Aleo (Varuna), and Tornado Cash (Groth16) all use proof systems with the formal ZK guarantee. STRK20s uses STARKs that are not formally ZK yet (Adrien confirmed). Monero’s Bulletproofs+ are formally ZK but only cover amount hiding; core sender privacy comes from ring signatures. Solana’s Bulletproofs are formally ZK but limited to range proofs. Zama uses FHE (different model). Canton uses access control (no ZK proofs).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Secretless</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
         <is>
           <t>users handle a single signing key (or none, via AA). no per-note secrets to manage or lose. STRK20s derives all keys from the Starknet account key via account abstraction. Aztec requires 3 separate key pairs. Aleo requires private key + view key. Railgun requires spending + viewing keys. Monero requires spend + view keys. Canton uses party keys managed via validator nodes. Others also require dedicated privacy key management.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Efficient note discovery</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>recipients discover funds in time proportional to their own activity. STRK20s uses on-chain indexed storage with shared secrets. Aztec uses a tagging mechanism but requires pre-registering senders. Zcash requires scanning all blocks and decrypting every transaction. Railgun and Aleo use standard record/UTXO scanning. Canton uses a ledger model, not applicable.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Compliance (viewing keys)</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>auditing entity can trace a specific user’s history without affecting others. STRK20s has third-party viewing keys. Zcash has full incoming/outgoing viewing keys. Aztec has incoming + outgoing viewing key pairs. Aleo has view keys plus Selective Disclosure and zPass for identity proofs. Railgun has scoped viewing keys (by block range) plus PPOI plus Koinly tax exports. Canton has sub-transaction privacy with full auditability and GDPR compliance built into Daml contracts (strongest institutional compliance story). Solana has auditor_elgamal_pubkey in mint config but feature is disabled. Monero has viewing keys but incoming only, all-or-nothing. Zama has programmable ACL contracts. Tornado Cash had a voluntary report tool only.</t>
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Selective disclosure</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>users can optionally reveal transaction history to a chosen third party (auditor, accountant, regulator, DAO) without affecting other users’ privacy. whether you use this for regulatory compliance, tax reporting, or governance is up to you. STRK20s has third-party viewing keys. Zcash has full incoming/outgoing viewing keys. Aztec has incoming + outgoing viewing key pairs. Aleo has view keys plus Selective Disclosure and zPass for identity proofs. Railgun has scoped viewing keys (by block range) plus PPOI plus Koinly tax exports. Canton has sub-transaction privacy with full auditability built into Daml contracts. Solana has auditor_elgamal_pubkey in mint config but feature is disabled. Monero has viewing keys but incoming only, all-or-nothing. Zama has programmable ACL contracts. Tornado Cash had a voluntary report tool only.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>CRYPTOGRAPHIC FOUNDATION</t>
         </is>
@@ -2690,43 +2834,43 @@
       <c r="B8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>No trusted setup</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>proof system requires no trusted setup ceremony. STARKs (Starknet) require none. Zcash Orchard uses Halo 2 (no setup) but Sapling pool still has one. Monero’s Bulletproofs+ and Solana’s ElGamal/Bulletproofs require none. Zama’s TFHE requires none. Canton doesn’t use ZK proofs, no ceremony needed. Aleo uses Varuna (Marlin-based universal SNARK) requiring a universal SRS. Aztec’s PLONK uses a universal updatable SRS (still a form of setup). Railgun and Tornado Cash use Groth16 requiring per-circuit ceremonies.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Post-quantum resistant</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>underlying cryptography resists quantum computing attacks. STARKs (hash-based) are post-quantum by design. Zama’s TFHE is lattice-based (LWE), considered PQ-resistant but less battle-tested. All SNARK/elliptic curve systems (Zcash, Aztec, Aleo, Railgun, Monero, Solana, Canton) are vulnerable to quantum attacks.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Succinct verifiability</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>anyone can verify chain integrity quickly and trustlessly on a small device. Enables rich client-side privacy proofs. ZK rollups (Starknet, Aztec) have this. L1s like Solana, Zcash, Monero, Aleo, and Canton do not. Aleo posts per-transaction proofs but doesn’t provide chain-level succinct state verification. Railgun runs on L1s without succinct verification.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>PERFORMANCE &amp; UX</t>
         </is>
@@ -2734,55 +2878,55 @@
       <c r="B12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Fast shield/unshield</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>how quickly a user can move between public and private states. measures the end-to-end time from initiating a shield (opt-in to privacy) or unshield (opt-out) to having usable funds. STRK20s: sub-2s block confirmation + sub-5s proof generation = seconds to shield or unshield. fastest of any protocol. Zcash: ~75s block time is the bottleneck. proof generation 2–5s but must wait for block confirmation. Monero: always private by default (instant opt-in), but no way to opt-out to a transparent state. Aztec: 36–72s block times in Alpha (targeting 3–4s by late 2026). Railgun: Ethereum block time (~12s) for the on-chain tx, but a mandatory 1-hour standby period after shielding before funds can be used (Private Proof of Innocence requirement). Tornado Cash: deposit was one Ethereum block, but real privacy required waiting hours for anonymity set to build. Aleo: off-chain proving but no concrete shielding speed benchmarks available. Solana: feature disabled on mainnet. Canton: access control model, no shielding concept. Zama: FHE operations are orders of magnitude slower than ZK.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Fast proof generation</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
-        <is>
-          <t>private transactions can be proved quickly on consumer hardware. STRK20s: Stwo prover targets sub-5-second client-side proving for full Cairo programs. Zcash: Orchard proofs take ~2–5s but only for simple shielded transfers. Aztec: PXE client-side proving works but proving times are still being optimized in Alpha. Aleo: client-side proving possible but resource-intensive; outsourceable to Prover Market. Railgun: Groth16 proving can be slow for complex circuits. Monero: ring signature computation is lightweight but not ZK. Zama: FHE is orders of magnitude slower than ZK. Canton, Solana: no ZK proving involved.</t>
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>End-to-end transaction time</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>end-to-end transaction time from user action to confirmed private transaction. the benchmark is Zcash Zashi: ~5 seconds on mobile, proof generated directly on the device. STRK20s: ~5 seconds end-to-end from the user’s perspective, but proof generation runs on the wallet operator backend (48-core machine), not on the user’s device. mobile proving is on the roadmap. for an apples-to-apples comparison, Zcash would also be faster if it ran proofs server-side. Aztec: PXE client-side proving works but proving times are still being optimized in Alpha. Aleo: client-side proving possible but resource-intensive; outsourceable to Prover Market. Railgun: Groth16 proving can be slow for complex circuits. Monero: ring signature computation is lightweight but not ZK. Zama: FHE is orders of magnitude slower than ZK. Canton, Solana: no ZK proving involved.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Scalable private transactions</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>high throughput and low cost for private operations specifically. Starknet: ~1,000 TPS today, targeting 10k+. sub-2s confirmation, $0.002 avg fee. Canton: claims no upper bound on TPS via horizontal scaling but access-control privacy model. Aleo: off-chain execution model is architecturally scalable but no composability between private apps limits real-world DeFi throughput. Zcash: PoW L1, ~75s blocks. Monero: PoW L1, 2-min blocks. Aztec: ~1 TPS in Alpha, 36–72s blocks. Railgun: inherits L1 gas costs. Solana: fast but privacy feature disabled. Zama: FHE is orders of magnitude slower. Tornado Cash: L1 gas costs.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t>Rich client-side proving</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>ability to prove complex logic (multi-calls, full smart contract execution, atomic DeFi operations) privately on the user’s device, verified cheaply on-chain. STRK20s: Cairo + Stwo prover enables proving entire Starknet block logic client-side. sub-5-second flow. Aztec: Noir + PXE executes private functions client-side in browser with ZK proofs. Aleo: Leo programs execute off-chain on client with ZK proofs, but no composability between private programs limits multi-step atomic operations. Zcash: limited to simple shielded transfers. Tornado Cash: “I have enough funds” was the ceiling. Railgun: bounded proof complexity. Solana: not succinctly verifiable. Zama: server-side FHE on coprocessors. Canton: no ZK proving, privacy via access control.</t>
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Programmable privacy</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>ability to prove complex logic (multi-calls, full smart contract execution, atomic DeFi operations) privately, verified cheaply on-chain. STRK20s: Cairo + Stwo enables proving entire Starknet block logic privately. atomic private AMM swaps (withdraw + swap + redeposit in one tx), account abstraction, session keys all work within the privacy layer. the highest ceiling of any privacy protocol. Aztec: Noir + PXE executes private functions in browser with ZK proofs. Aleo: Leo programs execute off-chain with ZK proofs, but no composability between private programs limits multi-step atomic operations. Zcash: limited to simple shielded transfers. Tornado Cash: “I have enough funds” was the ceiling. Railgun: bounded proof complexity. Solana: not succinctly verifiable. Zama: server-side FHE on coprocessors. Canton: no ZK proving, privacy via access control.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>ECOSYSTEM &amp; ACCESS</t>
         </is>
@@ -2790,60 +2934,60 @@
       <c r="B17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>DeFi composability</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>existing DeFi contracts require zero custom integration for private transactions. STRK20s and Railgun work with existing live protocols. Aztec and Canton have DeFi within their own ecosystems. Aleo has no composability between private applications (Equilibrium Labs: ‘one application can’t use the private state from another application as its input’). Zama and Solana require DeFi protocols to rewrite for encrypted types.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Existing ecosystem</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>live DeFi protocols, real liquidity, real users already present before privacy is added. Starknet, Zcash, Monero, Railgun (on Ethereum/Polygon/Arbitrum/BSC), Solana, and Canton ($4T annual tokenized volume, Goldman Sachs, HSBC, DTCC, Euroclear) all have established ecosystems. Aleo launched mainnet Sep 2024 and USDCx with Circle Jan 2026, but DeFi is still nascent. Aztec is in Alpha with no live DeFi. Zama’s ecosystem is nascent. Tornado Cash is OFAC-sanctioned.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>EVM compatible</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>privacy protocol runs on or integrates natively with EVM chains. Railgun operates as a smart contract on Ethereum, Polygon, Arbitrum, BSC. Tornado Cash was Ethereum-native. Zama’s fhEVM is an EVM-compatible confidential computing layer. STRK20s runs on Starknet (Cairo VM, not EVM). Aztec uses Noir. Aleo uses Leo. Zcash, Monero, Solana, Canton are all non-EVM chains.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Account abstraction</t>
         </is>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>privacy works with multisig, session keys, social recovery, smart accounts at the protocol level. STRK20s and Aztec both have native protocol-level AA. Monero has experimental CLI-only multisig via key splitting (not protocol-level). Aleo uses standard private key + view key + address model. Canton uses a party/validator model, not crypto-style AA. Others require standard key management.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>Hardware wallet support</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>users can secure private keys and sign privacy transactions with a hardware wallet. Starknet has Ledger support for standard transactions (via Ledger Live, Braavos, Argent X, and Ready multisig), but STRK20s privacy transactions are not yet available on hardware wallets. Monero: Ledger supports full shielded transactions. Zcash: Trezor supports Orchard shielded transactions, but Ledger supports transparent Zcash only. Solana: Ledger supports Solana, but confidential transfer feature is currently disabled on mainnet. Aztec, Aleo, Railgun, Zama, Canton, Tornado Cash: no hardware wallet integration for privacy features.</t>
         </is>
@@ -2909,42 +3053,42 @@
       <c r="I3" s="3" t="n"/>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>Protocol</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
         <is>
           <t>Private by
 design</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="34" t="inlineStr">
         <is>
           <t>Composable
 funds</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="34" t="inlineStr">
         <is>
           <t>Fast to
 use</t>
         </is>
       </c>
-      <c r="E4" s="32" t="inlineStr">
-        <is>
-          <t>Compliance
-ready</t>
-        </is>
-      </c>
-      <c r="F4" s="32" t="inlineStr">
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>Selective
+disclosure</t>
+        </is>
+      </c>
+      <c r="F4" s="34" t="inlineStr">
         <is>
           <t>Future-proof
 security</t>
         </is>
       </c>
-      <c r="G4" s="32" t="inlineStr">
+      <c r="G4" s="34" t="inlineStr">
         <is>
           <t>Wallet
 ready</t>
@@ -2954,38 +3098,38 @@
       <c r="I4" s="3" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="33" t="n"/>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="A5" s="35" t="n"/>
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>is my stuff
 actually private?</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C5" s="36" t="inlineStr">
         <is>
           <t>can I use
 private funds freely?</t>
         </is>
       </c>
-      <c r="D5" s="34" t="inlineStr">
+      <c r="D5" s="36" t="inlineStr">
         <is>
           <t>is the
 experience fast?</t>
         </is>
       </c>
-      <c r="E5" s="34" t="inlineStr">
+      <c r="E5" s="36" t="inlineStr">
         <is>
           <t>can institutions
 use this legally?</t>
         </is>
       </c>
-      <c r="F5" s="34" t="inlineStr">
+      <c r="F5" s="36" t="inlineStr">
         <is>
           <t>will this still be
 secure in 5 years?</t>
         </is>
       </c>
-      <c r="G5" s="34" t="inlineStr">
+      <c r="G5" s="36" t="inlineStr">
         <is>
           <t>does my
 wallet work?</t>
@@ -2995,37 +3139,37 @@
       <c r="I5" s="3" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>STRK20s (Starknet)</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C6" s="36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D6" s="36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E6" s="36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F6" s="36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G6" s="37" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G6" s="39" t="inlineStr">
         <is>
           <t>(✓)¹</t>
         </is>
@@ -3034,37 +3178,37 @@
       <c r="I6" s="3" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="38" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>Zcash</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>(✓)²</t>
         </is>
       </c>
-      <c r="C7" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D7" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E7" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F7" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G7" s="39" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E7" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
         <is>
           <t>(✓)³</t>
         </is>
@@ -3073,37 +3217,37 @@
       <c r="I7" s="3" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>Monero</t>
         </is>
       </c>
-      <c r="B8" s="43" t="inlineStr">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>(✓)⁴</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D8" s="43" t="inlineStr">
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>(✓)¹⁷</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E8" s="45" t="inlineStr">
         <is>
           <t>(✓)⁵</t>
         </is>
       </c>
-      <c r="F8" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G8" s="43" t="inlineStr">
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G8" s="45" t="inlineStr">
         <is>
           <t>(✓)⁶</t>
         </is>
@@ -3112,37 +3256,37 @@
       <c r="I8" s="3" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>Aztec</t>
         </is>
       </c>
-      <c r="B9" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C9" s="39" t="inlineStr">
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>(✓)⁷</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E9" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F9" s="39" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
         <is>
           <t>(✓)⁸</t>
         </is>
       </c>
-      <c r="G9" s="39" t="inlineStr">
+      <c r="G9" s="41" t="inlineStr">
         <is>
           <t>(✓)⁹</t>
         </is>
@@ -3151,37 +3295,37 @@
       <c r="I9" s="3" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>Aleo</t>
         </is>
       </c>
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>(✓)¹⁰</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D10" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E10" s="45" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F10" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G10" s="44" t="inlineStr">
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3190,37 +3334,37 @@
       <c r="I10" s="3" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>Railgun</t>
         </is>
       </c>
-      <c r="B11" s="39" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>(✓)¹¹</t>
         </is>
       </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D11" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E11" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F11" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G11" s="40" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G11" s="42" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3229,37 +3373,37 @@
       <c r="I11" s="3" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="42" t="inlineStr">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>Solana confidential</t>
         </is>
       </c>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C12" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D12" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E12" s="43" t="inlineStr">
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>(✓)¹²</t>
         </is>
       </c>
-      <c r="F12" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G12" s="44" t="inlineStr">
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G12" s="46" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3268,37 +3412,37 @@
       <c r="I12" s="3" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="38" t="inlineStr">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>Canton</t>
         </is>
       </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C13" s="39" t="inlineStr">
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>(✓)¹³</t>
         </is>
       </c>
-      <c r="D13" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E13" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F13" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G13" s="40" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E13" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G13" s="42" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3307,37 +3451,37 @@
       <c r="I13" s="3" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>Tornado Cash</t>
         </is>
       </c>
-      <c r="B14" s="43" t="inlineStr">
+      <c r="B14" s="45" t="inlineStr">
         <is>
           <t>(✓)¹⁵</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D14" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E14" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F14" s="44" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G14" s="44" t="inlineStr">
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G14" s="46" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3346,37 +3490,37 @@
       <c r="I14" s="3" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
         <is>
           <t>Zama (FHE)</t>
         </is>
       </c>
-      <c r="B15" s="39" t="inlineStr">
+      <c r="B15" s="41" t="inlineStr">
         <is>
           <t>(✓)¹⁶</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D15" s="40" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E15" s="41" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F15" s="39" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E15" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
         <is>
           <t>(✓)¹⁴</t>
         </is>
       </c>
-      <c r="G15" s="40" t="inlineStr">
+      <c r="G15" s="42" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3396,20 +3540,20 @@
       <c r="I16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>✓ = yes</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>(✓) = partially (see footnotes)</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
-      <c r="F17" s="25" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>– = no</t>
         </is>
@@ -3430,7 +3574,7 @@
       <c r="I18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>Footnotes</t>
         </is>
@@ -3445,7 +3589,7 @@
       <c r="I19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>¹  Starknet has full AA and wallet integration (Braavos, Argent), but STRK20s privacy transactions are not yet available on hardware wallets</t>
         </is>
@@ -3454,7 +3598,7 @@
       <c r="I20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>²  formally ZK proofs, but single-asset only (ZEC), no multi-asset pool, poor note discovery UX</t>
         </is>
@@ -3463,7 +3607,7 @@
       <c r="I21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>³  Trezor supports Orchard shielded transactions. Ledger only transparent</t>
         </is>
@@ -3472,7 +3616,7 @@
       <c r="I22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>⁴  always-on privacy with strongest anonymity set, but no multi-asset pool, no formal ZK proofs, no secretless design</t>
         </is>
@@ -3481,7 +3625,7 @@
       <c r="I23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>⁵  incoming viewing keys only. can’t reliably verify outgoing or balance</t>
         </is>
@@ -3490,7 +3634,7 @@
       <c r="I24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>⁶  Ledger supports full shielded transactions, but no account abstraction</t>
         </is>
@@ -3499,7 +3643,7 @@
       <c r="I25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>⁷  smart contracts exist but zero existing DeFi or liquidity. cold start problem</t>
         </is>
@@ -3508,7 +3652,7 @@
       <c r="I26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>⁸  PLONK uses universal SRS (still a setup). no post-quantum. but has succinct verifiability</t>
         </is>
@@ -3517,7 +3661,7 @@
       <c r="I27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="inlineStr">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>⁹  native AA, but no hardware wallet support for privacy transactions</t>
         </is>
@@ -3526,7 +3670,7 @@
       <c r="I28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>¹⁰  formally ZK but no multi-asset pool, no composability between private apps, no note discovery</t>
         </is>
@@ -3535,7 +3679,7 @@
       <c r="I29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>¹¹  formally ZK and multi-asset, but privacy limited by pool size per token. no client-side proving of complex logic</t>
         </is>
@@ -3544,7 +3688,7 @@
       <c r="I30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>¹²  auditor key exists in config but entire feature is disabled on mainnet</t>
         </is>
@@ -3553,7 +3697,7 @@
       <c r="I31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="inlineStr">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>¹³  DeFi within own Daml ecosystem only. requires separate smart contract language</t>
         </is>
@@ -3562,7 +3706,7 @@
       <c r="I32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="inlineStr">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>¹⁴  TFHE is lattice-based (PQ-resistant) and no trusted setup, but no succinct verifiability</t>
         </is>
@@ -3571,7 +3715,7 @@
       <c r="I33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="inlineStr">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>¹⁵  formally ZK (Groth16), but fragmented pools (fixed denominations), timing analysis could de-anonymize users, and protocol is OFAC-sanctioned/defunct</t>
         </is>
@@ -3580,7 +3724,7 @@
       <c r="I34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>¹⁶  FHE genuinely encrypts data during computation, but server-side model (not client-side ZK proofs). different trust model. ecosystem nascent</t>
         </is>
@@ -3589,7 +3733,7 @@
       <c r="I35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="inlineStr">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>¹⁷  privacy is always on so there’s no shielding step (zero friction to opt in). ~2 min block time for confirmations. seamless UX but slower than Starknet</t>
         </is>
@@ -3935,17 +4079,17 @@
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
       </c>
-      <c r="C4" s="46" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>Based on (from full Property Grid)</t>
         </is>
@@ -3954,36 +4098,36 @@
       <c r="E4" s="3" t="n"/>
     </row>
     <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="47" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Private by design</t>
         </is>
       </c>
-      <c r="B5" s="48" t="inlineStr">
+      <c r="B5" s="50" t="inlineStr">
         <is>
           <t>your balances, transfers, and identity are cryptographically hidden. the proof system itself guarantees no data leaks. you don’t manage separate secrets or scan the entire chain to find your funds.</t>
         </is>
       </c>
-      <c r="C5" s="49" t="inlineStr">
-        <is>
-          <t>multi-asset privacy pool + formally ZK proofs + secretless + efficient note discovery + rich client-side proving</t>
+      <c r="C5" s="51" t="inlineStr">
+        <is>
+          <t>multi-asset privacy pool + formally ZK proofs + secretless + efficient note discovery + programmable privacy</t>
         </is>
       </c>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
     </row>
     <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="52" t="inlineStr">
         <is>
           <t>Composable funds</t>
         </is>
       </c>
-      <c r="B6" s="51" t="inlineStr">
+      <c r="B6" s="53" t="inlineStr">
         <is>
           <t>your private funds can interact with live DeFi protocols (swap, lend, stake) without leaving the privacy layer or migrating to a new chain.</t>
         </is>
       </c>
-      <c r="C6" s="52" t="inlineStr">
+      <c r="C6" s="54" t="inlineStr">
         <is>
           <t>DeFi composability + existing ecosystem + EVM compatible</t>
         </is>
@@ -3992,55 +4136,55 @@
       <c r="E6" s="3" t="n"/>
     </row>
     <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>Fast to use</t>
         </is>
       </c>
-      <c r="B7" s="48" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>shielding (going private), unshielding (going public), and private transactions all happen in seconds. no waiting periods, no slow proof generation.</t>
         </is>
       </c>
-      <c r="C7" s="49" t="inlineStr">
-        <is>
-          <t>fast shield/unshield + fast proof generation + scalable private transactions</t>
+      <c r="C7" s="51" t="inlineStr">
+        <is>
+          <t>fast shield/unshield + end-to-end transaction time + scalable private transactions</t>
         </is>
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
     </row>
     <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="50" t="inlineStr">
-        <is>
-          <t>Compliance ready</t>
-        </is>
-      </c>
-      <c r="B8" s="51" t="inlineStr">
-        <is>
-          <t>institutions and regulated entities can use the protocol legally. selective disclosure lets auditors trace a specific user’s history without affecting anyone else’s privacy.</t>
-        </is>
-      </c>
-      <c r="C8" s="52" t="inlineStr">
-        <is>
-          <t>compliance (viewing keys)</t>
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>Selective disclosure</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>users can optionally reveal transaction history to a chosen third party (auditor, accountant, regulator, DAO) without affecting anyone else’s privacy.</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>selective disclosure</t>
         </is>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
     </row>
     <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>Future-proof security</t>
         </is>
       </c>
-      <c r="B9" s="48" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>the cryptographic foundation will still be secure when quantum computers arrive. no trusted setup ceremony that could be compromised. anyone can verify the chain on a small device.</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="51" t="inlineStr">
         <is>
           <t>no trusted setup + post-quantum proof system + succinct verifiability</t>
         </is>
@@ -4049,17 +4193,17 @@
       <c r="E9" s="3" t="n"/>
     </row>
     <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="50" t="inlineStr">
+      <c r="A10" s="52" t="inlineStr">
         <is>
           <t>Wallet ready</t>
         </is>
       </c>
-      <c r="B10" s="51" t="inlineStr">
+      <c r="B10" s="53" t="inlineStr">
         <is>
           <t>privacy works with your existing wallet setup: multisig, social recovery, session keys. hardware wallet signing is supported for the underlying chain.</t>
         </is>
       </c>
-      <c r="C10" s="52" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>account abstraction + hardware wallet support</t>
         </is>

</xml_diff>